<commit_message>
this is just a cleanup
</commit_message>
<xml_diff>
--- a/designs/user stories.xlsx
+++ b/designs/user stories.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/career/coursera/projects/global-produce/designs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D85409FD-8A90-364C-8EC1-EEC30E09A628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{225FBA30-1ADE-9146-8423-5975A864561F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="1800" windowWidth="28040" windowHeight="17440" xr2:uid="{2E0E2905-A103-4746-8E48-A7E12C7820A8}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19520" xr2:uid="{2E0E2905-A103-4746-8E48-A7E12C7820A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="79">
   <si>
     <t>ID</t>
   </si>
@@ -150,9 +150,6 @@
   </si>
   <si>
     <t>Log in to my account with verification</t>
-  </si>
-  <si>
-    <t>• Admin enters email and password.</t>
   </si>
   <si>
     <t>• Admin enters the verification code.</t>
@@ -379,30 +376,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">• System generates a verification code (saved at </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="8"/>
-        <rFont val="Arial Unicode MS"/>
-        <family val="2"/>
-      </rPr>
-      <t>Downloads/&lt;user_email&gt;/verification.txt</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="8"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">• If code is incorrect, show: </t>
     </r>
     <r>
@@ -641,13 +614,16 @@
       </rPr>
       <t>"No account found with the provided information. Please REGISTER"</t>
     </r>
+  </si>
+  <si>
+    <t>• System generates a verification code</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -747,12 +723,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="8"/>
-      <name val="Arial Unicode MS"/>
-      <family val="2"/>
     </font>
     <font>
       <i/>
@@ -818,23 +788,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1194,13 +1164,13 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D2" t="s">
@@ -1208,221 +1178,219 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
+      <c r="A3" s="8"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
       <c r="D3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
+      <c r="A4" s="8"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
       <c r="D4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
+      <c r="A5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
       <c r="D5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
+      <c r="A6" s="8"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
       <c r="D6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
       <c r="D7" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="5"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="18"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="18"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="11"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="13" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="11"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="13" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="18"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="13" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="18"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="16"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="11"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="13" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D13" s="10" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="16"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="16"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="8"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="10" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="8"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="10" t="s">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="16"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="8"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="10" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="8"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="10" t="s">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="16"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="8"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="10" t="s">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="16"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="8"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="10" t="s">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="13" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C20" s="6" t="s">
+      <c r="D20" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="12"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="7" t="s">
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="12"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="12"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="12"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="3" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="5"/>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="5"/>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="7" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="5"/>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="7" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="12"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="5"/>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="7" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="5"/>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="7" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="12"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="5"/>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="7" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="12"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="3" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="5"/>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="7" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -1433,196 +1401,196 @@
         <v>8</v>
       </c>
       <c r="C28" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="D28" s="6" t="s">
         <v>40</v>
-      </c>
-      <c r="D28" s="16" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="14"/>
       <c r="B29" s="15"/>
       <c r="C29" s="15"/>
-      <c r="D29" s="16" t="s">
-        <v>42</v>
+      <c r="D29" s="6" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="14"/>
       <c r="B30" s="15"/>
       <c r="C30" s="15"/>
-      <c r="D30" s="16" t="s">
-        <v>43</v>
+      <c r="D30" s="6" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="14"/>
       <c r="B31" s="15"/>
       <c r="C31" s="15"/>
-      <c r="D31" s="16" t="s">
+      <c r="D31" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" s="9" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C32" s="4" t="s">
+      <c r="D32" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="8"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="9"/>
+      <c r="D33" t="s">
         <v>45</v>
       </c>
-      <c r="D32" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="3"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" t="s">
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="8"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="9"/>
+      <c r="D34" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="3"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" t="s">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="8"/>
+      <c r="B35" s="9"/>
+      <c r="C35" s="9"/>
+      <c r="D35" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="3"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" t="s">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="8"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
+      <c r="D36" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="3"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" t="s">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="8"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="9"/>
+      <c r="D37" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="3"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" t="s">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="8"/>
+      <c r="B38" s="9"/>
+      <c r="C38" s="9"/>
+      <c r="D38" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="3"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" t="s">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C39" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="10"/>
+      <c r="B40" s="11"/>
+      <c r="C40" s="11"/>
+      <c r="D40" s="7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="B39" s="18" t="s">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="10"/>
+      <c r="B41" s="11"/>
+      <c r="C41" s="11"/>
+      <c r="D41" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="10"/>
+      <c r="B42" s="11"/>
+      <c r="C42" s="11"/>
+      <c r="D42" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="10"/>
+      <c r="B43" s="11"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B44" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C39" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="D39" s="19" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="17"/>
-      <c r="B40" s="18"/>
-      <c r="C40" s="18"/>
-      <c r="D40" s="19" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="17"/>
-      <c r="B41" s="18"/>
-      <c r="C41" s="18"/>
-      <c r="D41" s="19" t="s">
+      <c r="C44" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="12"/>
+      <c r="B45" s="13"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="12"/>
+      <c r="B46" s="13"/>
+      <c r="C46" s="13"/>
+      <c r="D46" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="17"/>
-      <c r="B42" s="18"/>
-      <c r="C42" s="18"/>
-      <c r="D42" s="19" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="17"/>
-      <c r="B43" s="18"/>
-      <c r="C43" s="18"/>
-      <c r="D43" s="19" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D44" s="7" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="5"/>
-      <c r="B45" s="6"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="7" t="s">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="12"/>
+      <c r="B47" s="13"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="5"/>
-      <c r="B46" s="6"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="5"/>
-      <c r="B47" s="6"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="7" t="s">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="12"/>
+      <c r="B48" s="13"/>
+      <c r="C48" s="13"/>
+      <c r="D48" s="3" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="5"/>
-      <c r="B48" s="6"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="7" t="s">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="12"/>
+      <c r="B49" s="13"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="3" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="5"/>
-      <c r="B49" s="6"/>
-      <c r="C49" s="6"/>
-      <c r="D49" s="7" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -1632,83 +1600,101 @@
       <c r="D50" s="2"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D51" t="s">
         <v>70</v>
       </c>
-      <c r="B51" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C51" s="4" t="s">
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="8"/>
+      <c r="B52" s="9"/>
+      <c r="C52" s="9"/>
+      <c r="D52" t="s">
         <v>71</v>
       </c>
-      <c r="D51" t="s">
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="8"/>
+      <c r="B53" s="9"/>
+      <c r="C53" s="9"/>
+      <c r="D53" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="3"/>
-      <c r="B52" s="4"/>
-      <c r="C52" s="4"/>
-      <c r="D52" t="s">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="8"/>
+      <c r="B54" s="9"/>
+      <c r="C54" s="9"/>
+      <c r="D54" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="3"/>
-      <c r="B53" s="4"/>
-      <c r="C53" s="4"/>
-      <c r="D53" t="s">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="8"/>
+      <c r="B55" s="9"/>
+      <c r="C55" s="9"/>
+      <c r="D55" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="3"/>
-      <c r="B54" s="4"/>
-      <c r="C54" s="4"/>
-      <c r="D54" t="s">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="8"/>
+      <c r="B56" s="9"/>
+      <c r="C56" s="9"/>
+      <c r="D56" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="3"/>
-      <c r="B55" s="4"/>
-      <c r="C55" s="4"/>
-      <c r="D55" t="s">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="8"/>
+      <c r="B57" s="9"/>
+      <c r="C57" s="9"/>
+      <c r="D57" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="3"/>
-      <c r="B56" s="4"/>
-      <c r="C56" s="4"/>
-      <c r="D56" t="s">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="8"/>
+      <c r="B58" s="9"/>
+      <c r="C58" s="9"/>
+      <c r="D58"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="8"/>
+      <c r="B59" s="9"/>
+      <c r="C59" s="9"/>
+      <c r="D59" t="s">
         <v>77</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="3"/>
-      <c r="B57" s="4"/>
-      <c r="C57" s="4"/>
-      <c r="D57" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="3"/>
-      <c r="B58" s="4"/>
-      <c r="C58" s="4"/>
-      <c r="D58"/>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="3"/>
-      <c r="B59" s="4"/>
-      <c r="C59" s="4"/>
-      <c r="D59" t="s">
-        <v>79</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="B8:B12"/>
+    <mergeCell ref="C8:C12"/>
+    <mergeCell ref="A2:A7"/>
+    <mergeCell ref="B2:B7"/>
+    <mergeCell ref="C2:C7"/>
+    <mergeCell ref="A32:A38"/>
+    <mergeCell ref="B32:B38"/>
+    <mergeCell ref="C32:C38"/>
+    <mergeCell ref="A13:A19"/>
+    <mergeCell ref="B13:B19"/>
+    <mergeCell ref="C13:C19"/>
+    <mergeCell ref="A20:A27"/>
+    <mergeCell ref="B20:B27"/>
+    <mergeCell ref="C20:C27"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="B28:B31"/>
+    <mergeCell ref="C28:C31"/>
     <mergeCell ref="A51:A59"/>
     <mergeCell ref="B51:B59"/>
     <mergeCell ref="C51:C59"/>
@@ -1718,24 +1704,6 @@
     <mergeCell ref="A44:A49"/>
     <mergeCell ref="B44:B49"/>
     <mergeCell ref="C44:C49"/>
-    <mergeCell ref="B20:B27"/>
-    <mergeCell ref="C20:C27"/>
-    <mergeCell ref="A28:A31"/>
-    <mergeCell ref="B28:B31"/>
-    <mergeCell ref="C28:C31"/>
-    <mergeCell ref="A32:A38"/>
-    <mergeCell ref="B32:B38"/>
-    <mergeCell ref="C32:C38"/>
-    <mergeCell ref="A13:A19"/>
-    <mergeCell ref="B13:B19"/>
-    <mergeCell ref="C13:C19"/>
-    <mergeCell ref="A20:A27"/>
-    <mergeCell ref="A8:A12"/>
-    <mergeCell ref="B8:B12"/>
-    <mergeCell ref="C8:C12"/>
-    <mergeCell ref="A2:A7"/>
-    <mergeCell ref="B2:B7"/>
-    <mergeCell ref="C2:C7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto PR: refactor/test-pr (#13)
* this is just a cleanup

* ci: use squash merge in auto pr workflow

---------

Co-authored-by: Shafi Hussein <inagurey.ahmed@gmail.com>
</commit_message>
<xml_diff>
--- a/designs/user stories.xlsx
+++ b/designs/user stories.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/career/coursera/projects/global-produce/designs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D85409FD-8A90-364C-8EC1-EEC30E09A628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{225FBA30-1ADE-9146-8423-5975A864561F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="1800" windowWidth="28040" windowHeight="17440" xr2:uid="{2E0E2905-A103-4746-8E48-A7E12C7820A8}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19520" xr2:uid="{2E0E2905-A103-4746-8E48-A7E12C7820A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="79">
   <si>
     <t>ID</t>
   </si>
@@ -150,9 +150,6 @@
   </si>
   <si>
     <t>Log in to my account with verification</t>
-  </si>
-  <si>
-    <t>• Admin enters email and password.</t>
   </si>
   <si>
     <t>• Admin enters the verification code.</t>
@@ -379,30 +376,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">• System generates a verification code (saved at </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="8"/>
-        <rFont val="Arial Unicode MS"/>
-        <family val="2"/>
-      </rPr>
-      <t>Downloads/&lt;user_email&gt;/verification.txt</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="8"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">• If code is incorrect, show: </t>
     </r>
     <r>
@@ -641,13 +614,16 @@
       </rPr>
       <t>"No account found with the provided information. Please REGISTER"</t>
     </r>
+  </si>
+  <si>
+    <t>• System generates a verification code</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -747,12 +723,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="8"/>
-      <name val="Arial Unicode MS"/>
-      <family val="2"/>
     </font>
     <font>
       <i/>
@@ -818,23 +788,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1194,13 +1164,13 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="9" t="s">
         <v>17</v>
       </c>
       <c r="D2" t="s">
@@ -1208,221 +1178,219 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
+      <c r="A3" s="8"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
       <c r="D3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
+      <c r="A4" s="8"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
       <c r="D4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
+      <c r="A5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
       <c r="D5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
+      <c r="A6" s="8"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
       <c r="D6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
       <c r="D7" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="5"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="18"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="18"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="11"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="13" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="11"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="13" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="18"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="13" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="18"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="16"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="11"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="13" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D13" s="10" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="16"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="16"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="8"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="10" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="8"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="10" t="s">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="16"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="8"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="10" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="8"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="10" t="s">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="16"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="8"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="10" t="s">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="16"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="8"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="10" t="s">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="13" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C20" s="6" t="s">
+      <c r="D20" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="12"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="7" t="s">
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="12"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="12"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="12"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="3" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="5"/>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="5"/>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="7" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="5"/>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="7" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="12"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="5"/>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="7" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="5"/>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="7" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="12"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="5"/>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="7" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="12"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="3" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="5"/>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="7" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -1433,196 +1401,196 @@
         <v>8</v>
       </c>
       <c r="C28" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="D28" s="6" t="s">
         <v>40</v>
-      </c>
-      <c r="D28" s="16" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="14"/>
       <c r="B29" s="15"/>
       <c r="C29" s="15"/>
-      <c r="D29" s="16" t="s">
-        <v>42</v>
+      <c r="D29" s="6" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="14"/>
       <c r="B30" s="15"/>
       <c r="C30" s="15"/>
-      <c r="D30" s="16" t="s">
-        <v>43</v>
+      <c r="D30" s="6" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="14"/>
       <c r="B31" s="15"/>
       <c r="C31" s="15"/>
-      <c r="D31" s="16" t="s">
+      <c r="D31" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" s="9" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C32" s="4" t="s">
+      <c r="D32" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="8"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="9"/>
+      <c r="D33" t="s">
         <v>45</v>
       </c>
-      <c r="D32" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="3"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" t="s">
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="8"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="9"/>
+      <c r="D34" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="3"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" t="s">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="8"/>
+      <c r="B35" s="9"/>
+      <c r="C35" s="9"/>
+      <c r="D35" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="3"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" t="s">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="8"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
+      <c r="D36" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="3"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" t="s">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="8"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="9"/>
+      <c r="D37" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="3"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" t="s">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="8"/>
+      <c r="B38" s="9"/>
+      <c r="C38" s="9"/>
+      <c r="D38" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="3"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" t="s">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C39" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="10"/>
+      <c r="B40" s="11"/>
+      <c r="C40" s="11"/>
+      <c r="D40" s="7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="B39" s="18" t="s">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="10"/>
+      <c r="B41" s="11"/>
+      <c r="C41" s="11"/>
+      <c r="D41" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="10"/>
+      <c r="B42" s="11"/>
+      <c r="C42" s="11"/>
+      <c r="D42" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="10"/>
+      <c r="B43" s="11"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B44" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C39" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="D39" s="19" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="17"/>
-      <c r="B40" s="18"/>
-      <c r="C40" s="18"/>
-      <c r="D40" s="19" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="17"/>
-      <c r="B41" s="18"/>
-      <c r="C41" s="18"/>
-      <c r="D41" s="19" t="s">
+      <c r="C44" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="12"/>
+      <c r="B45" s="13"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="12"/>
+      <c r="B46" s="13"/>
+      <c r="C46" s="13"/>
+      <c r="D46" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="17"/>
-      <c r="B42" s="18"/>
-      <c r="C42" s="18"/>
-      <c r="D42" s="19" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="17"/>
-      <c r="B43" s="18"/>
-      <c r="C43" s="18"/>
-      <c r="D43" s="19" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D44" s="7" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="5"/>
-      <c r="B45" s="6"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="7" t="s">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="12"/>
+      <c r="B47" s="13"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="5"/>
-      <c r="B46" s="6"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="5"/>
-      <c r="B47" s="6"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="7" t="s">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="12"/>
+      <c r="B48" s="13"/>
+      <c r="C48" s="13"/>
+      <c r="D48" s="3" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="5"/>
-      <c r="B48" s="6"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="7" t="s">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="12"/>
+      <c r="B49" s="13"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="3" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="5"/>
-      <c r="B49" s="6"/>
-      <c r="C49" s="6"/>
-      <c r="D49" s="7" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -1632,83 +1600,101 @@
       <c r="D50" s="2"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D51" t="s">
         <v>70</v>
       </c>
-      <c r="B51" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C51" s="4" t="s">
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="8"/>
+      <c r="B52" s="9"/>
+      <c r="C52" s="9"/>
+      <c r="D52" t="s">
         <v>71</v>
       </c>
-      <c r="D51" t="s">
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="8"/>
+      <c r="B53" s="9"/>
+      <c r="C53" s="9"/>
+      <c r="D53" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="3"/>
-      <c r="B52" s="4"/>
-      <c r="C52" s="4"/>
-      <c r="D52" t="s">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="8"/>
+      <c r="B54" s="9"/>
+      <c r="C54" s="9"/>
+      <c r="D54" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="3"/>
-      <c r="B53" s="4"/>
-      <c r="C53" s="4"/>
-      <c r="D53" t="s">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="8"/>
+      <c r="B55" s="9"/>
+      <c r="C55" s="9"/>
+      <c r="D55" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="3"/>
-      <c r="B54" s="4"/>
-      <c r="C54" s="4"/>
-      <c r="D54" t="s">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="8"/>
+      <c r="B56" s="9"/>
+      <c r="C56" s="9"/>
+      <c r="D56" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="3"/>
-      <c r="B55" s="4"/>
-      <c r="C55" s="4"/>
-      <c r="D55" t="s">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="8"/>
+      <c r="B57" s="9"/>
+      <c r="C57" s="9"/>
+      <c r="D57" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="3"/>
-      <c r="B56" s="4"/>
-      <c r="C56" s="4"/>
-      <c r="D56" t="s">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="8"/>
+      <c r="B58" s="9"/>
+      <c r="C58" s="9"/>
+      <c r="D58"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="8"/>
+      <c r="B59" s="9"/>
+      <c r="C59" s="9"/>
+      <c r="D59" t="s">
         <v>77</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="3"/>
-      <c r="B57" s="4"/>
-      <c r="C57" s="4"/>
-      <c r="D57" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="3"/>
-      <c r="B58" s="4"/>
-      <c r="C58" s="4"/>
-      <c r="D58"/>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="3"/>
-      <c r="B59" s="4"/>
-      <c r="C59" s="4"/>
-      <c r="D59" t="s">
-        <v>79</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="B8:B12"/>
+    <mergeCell ref="C8:C12"/>
+    <mergeCell ref="A2:A7"/>
+    <mergeCell ref="B2:B7"/>
+    <mergeCell ref="C2:C7"/>
+    <mergeCell ref="A32:A38"/>
+    <mergeCell ref="B32:B38"/>
+    <mergeCell ref="C32:C38"/>
+    <mergeCell ref="A13:A19"/>
+    <mergeCell ref="B13:B19"/>
+    <mergeCell ref="C13:C19"/>
+    <mergeCell ref="A20:A27"/>
+    <mergeCell ref="B20:B27"/>
+    <mergeCell ref="C20:C27"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="B28:B31"/>
+    <mergeCell ref="C28:C31"/>
     <mergeCell ref="A51:A59"/>
     <mergeCell ref="B51:B59"/>
     <mergeCell ref="C51:C59"/>
@@ -1718,24 +1704,6 @@
     <mergeCell ref="A44:A49"/>
     <mergeCell ref="B44:B49"/>
     <mergeCell ref="C44:C49"/>
-    <mergeCell ref="B20:B27"/>
-    <mergeCell ref="C20:C27"/>
-    <mergeCell ref="A28:A31"/>
-    <mergeCell ref="B28:B31"/>
-    <mergeCell ref="C28:C31"/>
-    <mergeCell ref="A32:A38"/>
-    <mergeCell ref="B32:B38"/>
-    <mergeCell ref="C32:C38"/>
-    <mergeCell ref="A13:A19"/>
-    <mergeCell ref="B13:B19"/>
-    <mergeCell ref="C13:C19"/>
-    <mergeCell ref="A20:A27"/>
-    <mergeCell ref="A8:A12"/>
-    <mergeCell ref="B8:B12"/>
-    <mergeCell ref="C8:C12"/>
-    <mergeCell ref="A2:A7"/>
-    <mergeCell ref="B2:B7"/>
-    <mergeCell ref="C2:C7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>